<commit_message>
Add PDF download script and update workbook with URL statuses
Co-authored-by: gladiola <17388845+gladiola@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/KandRStyle/research/references/Reference_Tracking.xlsx
+++ b/KandRStyle/research/references/Reference_Tracking.xlsx
@@ -472,7 +472,13 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at https://www.mybib.com/
+Call log:
+  - navigating to "https:/</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -488,7 +494,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at http://php.net/manual/en/security.database.sql-injection.ph</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -504,7 +514,13 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at https://owasp.org/index.php/Top
+Call log:
+  - navigating to</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -520,7 +536,13 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at https://www.scrt.ch/outils/mms/mms
+Call log:
+  - navigating</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -536,7 +558,13 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at https://www.youtube.com/watch?v=uK3
+Call log:
+  - navigatin</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -552,7 +580,13 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at https://www.scrt.ch/en/
+Call log:
+  - navigating to "https:</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -568,7 +602,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at https://www.nist.gov/news-events/events/2017/03/cybersecuri</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -584,7 +622,12 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at http://faculty.ucmerced.edu/wshadish/shadish-cv-jan-2015
+Ca</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -600,7 +643,13 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at http://faculty.ucmerced.edu/wshadish/biosketch
+Call log:
+  </t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -616,7 +665,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at http://www.ipr.northwestern.edu/workshops/annual-summer-wor</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -632,7 +685,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -648,7 +700,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -664,7 +715,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -680,7 +730,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -696,7 +745,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -712,7 +760,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -728,7 +775,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -744,7 +790,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -760,7 +805,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -776,7 +820,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -792,7 +835,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -808,7 +850,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -824,7 +865,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -840,7 +880,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -856,7 +895,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -872,7 +910,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -888,7 +925,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -904,7 +940,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -920,7 +955,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -936,7 +970,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -952,7 +985,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -968,7 +1000,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -984,7 +1015,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1000,7 +1030,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1016,7 +1045,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1032,7 +1060,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1048,7 +1075,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1064,7 +1090,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1080,7 +1105,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1096,7 +1120,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1112,7 +1135,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1128,7 +1150,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1144,7 +1165,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1160,7 +1180,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1176,7 +1195,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1192,7 +1210,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1208,7 +1225,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1224,7 +1240,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1240,7 +1255,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1256,7 +1270,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1272,7 +1285,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1288,7 +1300,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1304,7 +1315,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1320,7 +1330,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1336,7 +1345,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1352,7 +1360,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1368,7 +1375,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1384,7 +1390,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1400,7 +1405,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1416,7 +1420,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1432,7 +1435,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1448,7 +1450,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1464,7 +1465,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1480,7 +1480,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1496,7 +1495,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1512,7 +1510,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1528,7 +1525,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1544,7 +1540,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1560,7 +1555,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1576,7 +1570,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1592,7 +1585,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -1608,7 +1600,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1624,7 +1615,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -1640,7 +1630,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -1656,7 +1645,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -1672,7 +1660,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -1688,7 +1675,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -1704,7 +1690,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -1720,7 +1705,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -1736,7 +1720,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -1752,7 +1735,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -1768,7 +1750,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -1784,7 +1765,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -1800,7 +1780,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -1816,7 +1795,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -1832,7 +1810,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -1848,7 +1825,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -1864,7 +1840,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -1880,7 +1855,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -1896,7 +1870,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -1912,7 +1885,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -1928,7 +1900,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -1944,7 +1915,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -1960,7 +1930,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -1976,7 +1945,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -1992,7 +1960,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2008,7 +1975,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -2024,7 +1990,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -2040,7 +2005,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -2056,7 +2020,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -2072,7 +2035,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -2088,7 +2050,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -2104,7 +2065,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -2120,7 +2080,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -2136,7 +2095,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -2152,7 +2110,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -2168,7 +2125,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -2184,7 +2140,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -2200,7 +2155,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -2216,7 +2170,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -2232,7 +2185,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -2248,7 +2200,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -2264,7 +2215,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -2280,7 +2230,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -2296,7 +2245,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -2312,7 +2260,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -2328,7 +2275,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -2344,7 +2290,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -2360,7 +2305,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -2376,7 +2320,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -2392,7 +2335,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -2408,7 +2350,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -2424,7 +2365,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -2440,7 +2380,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -2456,7 +2395,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -2472,7 +2410,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -2488,7 +2425,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -2504,7 +2440,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -2520,7 +2455,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -2536,7 +2470,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -2552,7 +2485,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -2568,7 +2500,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -2584,7 +2515,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -2600,7 +2530,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -2616,7 +2545,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -2632,7 +2560,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -2648,7 +2575,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -2664,7 +2590,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -2680,7 +2605,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -2696,7 +2620,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -2712,7 +2635,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -2728,7 +2650,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -2744,7 +2665,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -2760,7 +2680,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -2776,7 +2695,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -2792,7 +2710,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -2808,7 +2725,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -2824,7 +2740,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -2840,7 +2755,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -2856,7 +2770,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -2872,7 +2785,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -2888,7 +2800,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -2904,7 +2815,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -2920,7 +2830,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -2936,7 +2845,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -2952,7 +2860,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -2968,7 +2875,6 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix path duplicity - use relative paths in scripts
Co-authored-by: gladiola <17388845+gladiola@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/KandRStyle/research/references/Reference_Tracking.xlsx
+++ b/KandRStyle/research/references/Reference_Tracking.xlsx
@@ -472,13 +472,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at https://www.mybib.com/
-Call log:
-  - navigating to "https:/</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -494,11 +488,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at http://php.net/manual/en/security.database.sql-injection.ph</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -514,13 +504,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at https://owasp.org/index.php/Top
-Call log:
-  - navigating to</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -536,13 +520,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at https://www.scrt.ch/outils/mms/mms
-Call log:
-  - navigating</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -558,13 +536,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at https://www.youtube.com/watch?v=uK3
-Call log:
-  - navigatin</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -580,13 +552,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at https://www.scrt.ch/en/
-Call log:
-  - navigating to "https:</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -602,11 +568,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at https://www.nist.gov/news-events/events/2017/03/cybersecuri</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -622,12 +584,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at http://faculty.ucmerced.edu/wshadish/shadish-cv-jan-2015
-Ca</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -643,13 +600,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at http://faculty.ucmerced.edu/wshadish/biosketch
-Call log:
-  </t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -665,11 +616,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at http://www.ipr.northwestern.edu/workshops/annual-summer-wor</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -685,6 +632,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -700,6 +648,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -715,6 +664,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -730,6 +680,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -745,6 +696,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -760,6 +712,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -775,6 +728,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -790,6 +744,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -805,6 +760,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -820,6 +776,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -835,6 +792,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -850,6 +808,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -865,6 +824,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -880,6 +840,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -895,6 +856,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -910,6 +872,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -925,6 +888,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -940,6 +904,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -955,6 +920,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -970,6 +936,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -985,6 +952,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1000,6 +968,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1015,6 +984,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1030,6 +1000,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1045,6 +1016,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1060,6 +1032,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1075,6 +1048,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1090,6 +1064,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1105,6 +1080,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1120,6 +1096,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1135,6 +1112,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1150,6 +1128,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1165,6 +1144,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1180,6 +1160,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1195,6 +1176,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1210,6 +1192,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1225,6 +1208,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1240,6 +1224,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1255,6 +1240,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1270,6 +1256,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1285,6 +1272,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1300,6 +1288,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1315,6 +1304,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1330,6 +1320,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1345,6 +1336,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1360,6 +1352,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1375,6 +1368,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1390,6 +1384,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1405,6 +1400,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1420,6 +1416,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1435,6 +1432,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1450,6 +1448,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1465,6 +1464,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1480,6 +1480,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1495,6 +1496,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1510,6 +1512,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1525,6 +1528,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1540,6 +1544,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1555,6 +1560,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1570,6 +1576,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1585,6 +1592,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -1600,6 +1608,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1615,6 +1624,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -1630,6 +1640,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -1645,6 +1656,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -1660,6 +1672,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -1675,6 +1688,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -1690,6 +1704,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -1705,6 +1720,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -1720,6 +1736,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -1735,6 +1752,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -1750,6 +1768,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -1765,6 +1784,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -1780,6 +1800,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -1795,6 +1816,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -1810,6 +1832,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -1825,6 +1848,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -1840,6 +1864,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -1855,6 +1880,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -1870,6 +1896,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -1885,6 +1912,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -1900,6 +1928,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -1915,6 +1944,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -1930,6 +1960,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -1945,6 +1976,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -1960,6 +1992,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -1975,6 +2008,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -1990,6 +2024,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -2005,6 +2040,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -2020,6 +2056,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -2035,6 +2072,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -2050,6 +2088,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -2065,6 +2104,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -2080,6 +2120,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -2095,6 +2136,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -2110,6 +2152,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -2125,6 +2168,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -2140,6 +2184,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -2155,6 +2200,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -2170,6 +2216,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -2185,6 +2232,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -2200,6 +2248,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -2215,6 +2264,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -2230,6 +2280,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -2245,6 +2296,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -2260,6 +2312,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -2275,6 +2328,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -2290,6 +2344,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -2305,6 +2360,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -2320,6 +2376,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -2335,6 +2392,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -2350,6 +2408,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -2365,6 +2424,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -2380,6 +2440,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -2395,6 +2456,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -2410,6 +2472,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -2425,6 +2488,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -2440,6 +2504,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -2455,6 +2520,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -2470,6 +2536,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -2485,6 +2552,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -2500,6 +2568,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -2515,6 +2584,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -2530,6 +2600,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -2545,6 +2616,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -2560,6 +2632,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -2575,6 +2648,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -2590,6 +2664,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -2605,6 +2680,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -2620,6 +2696,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -2635,6 +2712,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -2650,6 +2728,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -2665,6 +2744,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -2680,6 +2760,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -2695,6 +2776,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -2710,6 +2792,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -2725,6 +2808,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -2740,6 +2824,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -2755,6 +2840,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -2770,6 +2856,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -2785,6 +2872,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -2800,6 +2888,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -2815,6 +2904,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -2830,6 +2920,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -2845,6 +2936,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -2860,6 +2952,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -2875,6 +2968,7 @@
           <t>Not Found</t>
         </is>
       </c>
+      <c r="D158" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Accessed Date column to workbook and improve Wayback integration
Co-authored-by: gladiola <17388845+gladiola@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/KandRStyle/research/references/Reference_Tracking.xlsx
+++ b/KandRStyle/research/references/Reference_Tracking.xlsx
@@ -427,13 +427,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D158"/>
+  <dimension ref="A1:E158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,10 +450,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Accessed Date</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -469,10 +475,15 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>12 July 2026</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -483,12 +494,13 @@
           <t>http://php.net/manual/en/security.database.sql-injection.php</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -499,12 +511,13 @@
           <t>https://owasp.org/index.php/Top</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -515,12 +528,13 @@
           <t>https://www.scrt.ch/outils/mms/mms</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -531,12 +545,13 @@
           <t>https://www.youtube.com/watch?v=uK3</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -547,12 +562,13 @@
           <t>https://www.scrt.ch/en/</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -563,12 +579,13 @@
           <t>https://www.nist.gov/news-events/events/2017/03/cybersecurity-framework-virtual-events</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -579,12 +596,13 @@
           <t>http://faculty.ucmerced.edu/wshadish/shadish-cv-jan-2015</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -595,12 +613,13 @@
           <t>http://faculty.ucmerced.edu/wshadish/biosketch</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -611,12 +630,13 @@
           <t>http://www.ipr.northwestern.edu/workshops/annual-summer-workshops/quasi-experimental-design-and-analysis/</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -627,12 +647,13 @@
           <t>https://www.kali.org/</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -643,12 +664,13 @@
           <t>https://www.virtualbox.org/</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -659,12 +681,13 @@
           <t>http://www.vmware.com/</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -675,12 +698,13 @@
           <t>https://azure.microsoft.com/en-us/?cdn=disable</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -691,12 +715,13 @@
           <t>http://junit.org/junit4/</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -707,12 +732,13 @@
           <t>http://qunitjs.com/</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -723,12 +749,13 @@
           <t>https://phpunit.de/</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -739,12 +766,13 @@
           <t>http://docs.seleniumhq.org/</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -755,12 +783,13 @@
           <t>https://www.microsoft.com/en-us/download/details.aspx?id=3702</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -771,12 +800,13 @@
           <t>https://www.mysql.com/</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -787,12 +817,13 @@
           <t>https://www.phpmyadmin.net/</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -803,12 +834,13 @@
           <t>http://192.168.56.101/chapter4example.exe</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -819,12 +851,13 @@
           <t>https://www.owasp.org/index.php/File:Automated-</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -835,12 +868,13 @@
           <t>http://searchsecurity.techtarget.com/opinion/Wendy-Nather-Were-on-a-trajectory-for-profound-change</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -851,12 +885,13 @@
           <t>http://insecure.org/stf/smashstack.html</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -867,12 +902,13 @@
           <t>http://www.primalsecurity.net/0x0-</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -883,12 +919,13 @@
           <t>https://www.raspberrypi.org/downloads/raspbian/</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -899,12 +936,13 @@
           <t>https://docs.kali.org/kali-on-arm/install-kali-linux-arm-raspberry-pi</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -915,12 +953,13 @@
           <t>https://docs.microsoft.com/en-us/powershell/module/microsoft.powershell.utility/get-filehash?view=powershell-5.1</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -931,12 +970,13 @@
           <t>https://unix.stackexchange.com/questions/151547/linux-set-date-through-command-line</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -947,12 +987,13 @@
           <t>https://www.aircrack-ng.org/</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -963,12 +1004,13 @@
           <t>https://www.aircrack-ng.org/doku.php?id=compatibility</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -979,12 +1021,13 @@
           <t>https://wikidevi.com/wiki/TP-LINK</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -995,12 +1038,13 @@
           <t>https://wikidevi.com/wiki/ALFA</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1011,12 +1055,13 @@
           <t>https://hakshop.com/products/wifi-pineappling-book</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1027,12 +1072,13 @@
           <t>http://goo.gl/iMVWew</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1043,12 +1089,13 @@
           <t>https://www.raspberrypi.org/</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1059,12 +1106,13 @@
           <t>https://www.raspberrypi.org/documentation/</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1075,12 +1123,13 @@
           <t>https://www.walmart.com/ip/TP-LINK-TL-WN722N-N150-High-Gain-Wireless-USB-Adapter/17133249</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1091,12 +1140,13 @@
           <t>https://www.amazon.com/Alfa-AWUS036NH-802-11g-Wireless-Long-Range/dp/B003YIFHJY</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1107,12 +1157,13 @@
           <t>https://www.amazon.com/Alfa-AWUSO36NH-Wireless-Long-Rang-Network/dp/B0035APGP6</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1123,12 +1174,13 @@
           <t>https://www.csoonline.com/article/2462478/microsoft-subnet/hacker-hunts-and-pwns-wifi-pineapples-with-0-day-at-def-con.html</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1139,12 +1191,13 @@
           <t>https://twitter.com/ihuntpineapples/media</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1155,12 +1208,13 @@
           <t>https://www.reddit.com/r/Defcon/comments/2d16lk/your</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1171,12 +1225,13 @@
           <t>https://capec.mitre.org/</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1187,12 +1242,13 @@
           <t>https://capec.mitre.org/data/definitions/1000.html</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1203,12 +1259,13 @@
           <t>https://capec.mitre.org/data/definitions/152.html</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1219,12 +1276,13 @@
           <t>https://capec.mitre.org/data/definitions/137.html</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1235,12 +1293,13 @@
           <t>https://capec.mitre.org/data/definitions/513.html</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1251,12 +1310,13 @@
           <t>https://capec.mitre.org/data/definitions/248.html</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1267,12 +1327,13 @@
           <t>https://capec.mitre.org/data/definitions/66.html</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1283,12 +1344,13 @@
           <t>https://capec.mitre.org/data/definitions/108.html</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1299,12 +1361,13 @@
           <t>http://cwe.mitre.org/data/definitions/707.html</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1315,12 +1378,13 @@
           <t>http://cwe.mitre.org/data/definitions/74.html</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1331,12 +1395,13 @@
           <t>http://capec.mitre.org/data/definitions/242.html</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1347,12 +1412,13 @@
           <t>https://capec.mitre.org/data/definitions/110.html</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1363,12 +1429,13 @@
           <t>http://cwe.mitre.org/data/definitions/89.html</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1379,12 +1446,13 @@
           <t>http://cwe.mitre.org/data/definitions/929.html</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1397,10 +1465,15 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
+          <t>4 Aug 2026</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1411,12 +1484,13 @@
           <t>https://fred.stlouisfed.org/series/POPTOTASA647NWDB</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1427,12 +1501,13 @@
           <t>https://www.census.gov/quickfacts/chattanoogacitytennessee</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr"/>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1443,12 +1518,13 @@
           <t>https://www.census.gov/quickfacts/fact/table/TN/PST045222</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1459,12 +1535,13 @@
           <t>https://fred.stlouisfed.org/series/CAPOP</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1475,12 +1552,13 @@
           <t>https://www2.census.gov/programs-surveys/popest/datasets/2020-2022/state/totals/NST-EST2022-POPCHG2020_2022.csv</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr"/>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1491,12 +1569,13 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2016State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1507,12 +1586,13 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2016_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1523,12 +1603,13 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2017State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1539,12 +1620,13 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2017_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1555,12 +1637,13 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2018State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1571,12 +1654,13 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2018_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1587,12 +1671,13 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2019State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -1603,12 +1688,13 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2019_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr"/>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1619,12 +1705,13 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2020State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr"/>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -1635,12 +1722,13 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2020_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr"/>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -1651,12 +1739,13 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2021State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -1667,12 +1756,13 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2021_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -1683,12 +1773,13 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2022State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr"/>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -1699,12 +1790,13 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2022_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr"/>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -1717,10 +1809,15 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -1733,10 +1830,15 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -1749,10 +1851,15 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -1765,10 +1872,15 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -1781,10 +1893,15 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -1797,10 +1914,15 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -1813,10 +1935,15 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -1829,10 +1956,15 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -1845,10 +1977,15 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -1861,10 +1998,15 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -1877,10 +2019,15 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -1893,10 +2040,15 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -1909,10 +2061,15 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -1925,10 +2082,15 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -1941,10 +2103,15 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -1957,10 +2124,15 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -1973,10 +2145,15 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -1989,10 +2166,15 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2005,10 +2187,15 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -2021,10 +2208,15 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -2037,10 +2229,15 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -2053,10 +2250,15 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -2069,10 +2271,15 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -2085,10 +2292,15 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -2101,10 +2313,15 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -2117,10 +2334,15 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -2133,10 +2355,15 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -2149,10 +2376,15 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -2165,10 +2397,15 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -2181,10 +2418,15 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -2197,10 +2439,15 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -2213,10 +2460,15 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -2229,10 +2481,15 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -2245,10 +2502,15 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -2261,10 +2523,15 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -2277,10 +2544,15 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -2293,10 +2565,15 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -2309,10 +2586,15 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -2325,10 +2607,15 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -2341,10 +2628,15 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -2357,10 +2649,15 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -2373,10 +2670,15 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -2389,10 +2691,15 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -2405,10 +2712,15 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -2421,10 +2733,15 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -2437,10 +2754,15 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -2453,10 +2775,15 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -2469,10 +2796,15 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -2485,10 +2817,15 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -2501,10 +2838,15 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -2517,10 +2859,15 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -2533,10 +2880,15 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -2549,10 +2901,15 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -2565,10 +2922,15 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -2581,10 +2943,15 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -2597,10 +2964,15 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -2613,10 +2985,15 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -2629,10 +3006,15 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -2645,10 +3027,15 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -2661,10 +3048,15 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -2677,10 +3069,15 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -2693,10 +3090,15 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr"/>
+          <t>21 June 2026</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -2709,10 +3111,15 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr"/>
+          <t>12 July 2026</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -2725,10 +3132,15 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr"/>
+          <t>12 July 2026</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -2741,10 +3153,15 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr"/>
+          <t>12 July 2026</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -2757,10 +3174,15 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr"/>
+          <t>12 July 2026</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -2773,10 +3195,15 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr"/>
+          <t>13 July 2026</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -2787,12 +3214,13 @@
           <t>https://doi.org/10.6028/nist.sp.800-88r2</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr"/>
+      <c r="C147" t="inlineStr"/>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -2803,12 +3231,13 @@
           <t>https://theretroweb.com/storage/documentation/wd6000-velociraptor-68407cb5c0c96653507203.pdf</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr"/>
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -2819,12 +3248,13 @@
           <t>https://www.cyberciti.biz/faq/create-a-freebsd-swap-file/</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr"/>
+      <c r="C149" t="inlineStr"/>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -2835,12 +3265,13 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=enc</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr"/>
+      <c r="C150" t="inlineStr"/>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -2851,12 +3282,13 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=zfs</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr"/>
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -2867,12 +3299,13 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=zpool</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr"/>
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -2883,12 +3316,13 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=geom</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr"/>
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -2899,12 +3333,13 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=geli</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr"/>
+      <c r="C154" t="inlineStr"/>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -2915,12 +3350,13 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=gpart</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr"/>
+      <c r="C155" t="inlineStr"/>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -2931,12 +3367,13 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=dd</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr"/>
+      <c r="C156" t="inlineStr"/>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -2947,12 +3384,13 @@
           <t>https://docs.freebsd.org/en/books/handbook/zfs/</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr"/>
+      <c r="C157" t="inlineStr"/>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -2963,12 +3401,13 @@
           <t>https://docs.freebsd.org/en/books/handbook/disks/</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>Not Found</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr"/>
+      <c r="C158" t="inlineStr"/>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
trying a reference pull-down scraping script.  Many of the references are too old to be effective anymore.
</commit_message>
<xml_diff>
--- a/KandRStyle/research/references/Reference_Tracking.xlsx
+++ b/KandRStyle/research/references/Reference_Tracking.xlsx
@@ -475,7 +475,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>12 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -483,7 +483,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -494,13 +498,21 @@
           <t>http://php.net/manual/en/security.database.sql-injection.php</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -511,13 +523,21 @@
           <t>https://owasp.org/index.php/Top</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -528,13 +548,21 @@
           <t>https://www.scrt.ch/outils/mms/mms</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -545,13 +573,21 @@
           <t>https://www.youtube.com/watch?v=uK3</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -562,13 +598,21 @@
           <t>https://www.scrt.ch/en/</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -579,13 +623,21 @@
           <t>https://www.nist.gov/news-events/events/2017/03/cybersecurity-framework-virtual-events</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -596,13 +648,21 @@
           <t>http://faculty.ucmerced.edu/wshadish/shadish-cv-jan-2015</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -613,13 +673,21 @@
           <t>http://faculty.ucmerced.edu/wshadish/biosketch</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -630,13 +698,21 @@
           <t>http://www.ipr.northwestern.edu/workshops/annual-summer-workshops/quasi-experimental-design-and-analysis/</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -647,13 +723,21 @@
           <t>https://www.kali.org/</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -664,13 +748,21 @@
           <t>https://www.virtualbox.org/</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -681,13 +773,21 @@
           <t>http://www.vmware.com/</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -698,13 +798,21 @@
           <t>https://azure.microsoft.com/en-us/?cdn=disable</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -715,13 +823,21 @@
           <t>http://junit.org/junit4/</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -732,13 +848,21 @@
           <t>http://qunitjs.com/</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -749,13 +873,21 @@
           <t>https://phpunit.de/</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -766,13 +898,21 @@
           <t>http://docs.seleniumhq.org/</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -783,13 +923,21 @@
           <t>https://www.microsoft.com/en-us/download/details.aspx?id=3702</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -800,13 +948,21 @@
           <t>https://www.mysql.com/</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -817,13 +973,21 @@
           <t>https://www.phpmyadmin.net/</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -834,13 +998,21 @@
           <t>http://192.168.56.101/chapter4example.exe</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Local/private URL - cannot archive</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -851,13 +1023,21 @@
           <t>https://www.owasp.org/index.php/File:Automated-</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -868,13 +1048,21 @@
           <t>http://searchsecurity.techtarget.com/opinion/Wendy-Nather-Were-on-a-trajectory-for-profound-change</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -885,13 +1073,21 @@
           <t>http://insecure.org/stf/smashstack.html</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -902,13 +1098,21 @@
           <t>http://www.primalsecurity.net/0x0-</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -919,13 +1123,21 @@
           <t>https://www.raspberrypi.org/downloads/raspbian/</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -936,13 +1148,21 @@
           <t>https://docs.kali.org/kali-on-arm/install-kali-linux-arm-raspberry-pi</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -953,13 +1173,21 @@
           <t>https://docs.microsoft.com/en-us/powershell/module/microsoft.powershell.utility/get-filehash?view=powershell-5.1</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -970,13 +1198,21 @@
           <t>https://unix.stackexchange.com/questions/151547/linux-set-date-through-command-line</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -987,13 +1223,21 @@
           <t>https://www.aircrack-ng.org/</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1004,13 +1248,21 @@
           <t>https://www.aircrack-ng.org/doku.php?id=compatibility</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1021,13 +1273,21 @@
           <t>https://wikidevi.com/wiki/TP-LINK</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1038,13 +1298,21 @@
           <t>https://wikidevi.com/wiki/ALFA</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1055,13 +1323,21 @@
           <t>https://hakshop.com/products/wifi-pineappling-book</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1072,13 +1348,21 @@
           <t>http://goo.gl/iMVWew</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1089,13 +1373,21 @@
           <t>https://www.raspberrypi.org/</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1106,13 +1398,21 @@
           <t>https://www.raspberrypi.org/documentation/</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1123,13 +1423,21 @@
           <t>https://www.walmart.com/ip/TP-LINK-TL-WN722N-N150-High-Gain-Wireless-USB-Adapter/17133249</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1140,13 +1448,21 @@
           <t>https://www.amazon.com/Alfa-AWUS036NH-802-11g-Wireless-Long-Range/dp/B003YIFHJY</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1157,13 +1473,21 @@
           <t>https://www.amazon.com/Alfa-AWUSO36NH-Wireless-Long-Rang-Network/dp/B0035APGP6</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1174,13 +1498,21 @@
           <t>https://www.csoonline.com/article/2462478/microsoft-subnet/hacker-hunts-and-pwns-wifi-pineapples-with-0-day-at-def-con.html</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1191,13 +1523,21 @@
           <t>https://twitter.com/ihuntpineapples/media</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1208,13 +1548,21 @@
           <t>https://www.reddit.com/r/Defcon/comments/2d16lk/your</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D45" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1225,13 +1573,21 @@
           <t>https://capec.mitre.org/</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D46" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1242,13 +1598,21 @@
           <t>https://capec.mitre.org/data/definitions/1000.html</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D47" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1259,13 +1623,21 @@
           <t>https://capec.mitre.org/data/definitions/152.html</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D48" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1276,13 +1648,21 @@
           <t>https://capec.mitre.org/data/definitions/137.html</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1293,13 +1673,21 @@
           <t>https://capec.mitre.org/data/definitions/513.html</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D50" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1310,13 +1698,21 @@
           <t>https://capec.mitre.org/data/definitions/248.html</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D51" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1327,13 +1723,21 @@
           <t>https://capec.mitre.org/data/definitions/66.html</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D52" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1344,13 +1748,21 @@
           <t>https://capec.mitre.org/data/definitions/108.html</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D53" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1361,13 +1773,21 @@
           <t>http://cwe.mitre.org/data/definitions/707.html</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1378,13 +1798,21 @@
           <t>http://cwe.mitre.org/data/definitions/74.html</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D55" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1395,13 +1823,21 @@
           <t>http://capec.mitre.org/data/definitions/242.html</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D56" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1412,13 +1848,21 @@
           <t>https://capec.mitre.org/data/definitions/110.html</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D57" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1429,13 +1873,21 @@
           <t>http://cwe.mitre.org/data/definitions/89.html</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D58" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1446,13 +1898,21 @@
           <t>http://cwe.mitre.org/data/definitions/929.html</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1465,7 +1925,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>4 Aug 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1473,7 +1933,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1484,13 +1948,21 @@
           <t>https://fred.stlouisfed.org/series/POPTOTASA647NWDB</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1501,13 +1973,21 @@
           <t>https://www.census.gov/quickfacts/chattanoogacitytennessee</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D62" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1518,13 +1998,21 @@
           <t>https://www.census.gov/quickfacts/fact/table/TN/PST045222</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D63" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1535,13 +2023,21 @@
           <t>https://fred.stlouisfed.org/series/CAPOP</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D64" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1552,13 +2048,21 @@
           <t>https://www2.census.gov/programs-surveys/popest/datasets/2020-2022/state/totals/NST-EST2022-POPCHG2020_2022.csv</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D65" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1569,13 +2073,21 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2016State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D66" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1586,13 +2098,21 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2016_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D67" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1603,13 +2123,21 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2017State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D68" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1620,13 +2148,21 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2017_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D69" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1637,13 +2173,21 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2018State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D70" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1654,13 +2198,21 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2018_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D71" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1671,13 +2223,21 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2019State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D72" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -1688,13 +2248,21 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2019_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D73" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1705,13 +2273,21 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2020State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D74" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -1722,13 +2298,21 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2020_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D75" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -1739,13 +2323,21 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2021State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D76" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -1756,13 +2348,21 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2021_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D77" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -1773,13 +2373,21 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2022State/StateReport.aspx</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D78" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -1790,13 +2398,21 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2022_IC3Report.pdf</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D79" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -1809,7 +2425,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -1817,7 +2433,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -1830,7 +2450,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -1838,7 +2458,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -1851,7 +2475,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -1859,7 +2483,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -1872,7 +2500,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -1880,7 +2508,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -1893,7 +2525,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -1901,7 +2533,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -1914,7 +2550,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -1922,7 +2558,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -1935,7 +2575,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -1943,7 +2583,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -1956,7 +2600,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -1964,7 +2608,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -1977,7 +2625,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -1985,7 +2633,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -1998,7 +2650,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2006,7 +2658,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -2019,7 +2675,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2027,7 +2683,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -2040,7 +2700,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2048,7 +2708,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -2061,7 +2725,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2069,7 +2733,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -2082,7 +2750,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2090,7 +2758,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -2103,7 +2775,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2111,7 +2783,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -2124,7 +2800,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2132,7 +2808,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -2145,7 +2825,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2153,7 +2833,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -2166,7 +2850,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2174,7 +2858,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2187,7 +2875,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2195,7 +2883,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -2208,7 +2900,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2216,7 +2908,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -2229,7 +2925,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2237,7 +2933,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -2250,7 +2950,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2258,7 +2958,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -2271,7 +2975,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2279,7 +2983,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -2292,7 +3000,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2300,7 +3008,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -2313,7 +3025,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2321,7 +3033,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -2334,7 +3050,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2342,7 +3058,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -2355,7 +3075,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -2363,7 +3083,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -2376,7 +3100,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -2384,7 +3108,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -2397,7 +3125,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -2405,7 +3133,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -2418,7 +3150,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -2426,7 +3158,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -2439,7 +3175,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -2447,7 +3183,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -2460,7 +3200,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -2468,7 +3208,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -2481,7 +3225,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -2489,7 +3233,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -2502,7 +3250,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -2510,7 +3258,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -2523,7 +3275,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -2531,7 +3283,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -2544,7 +3300,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -2552,7 +3308,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -2565,7 +3325,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -2573,7 +3333,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -2586,7 +3350,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -2594,7 +3358,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -2607,7 +3375,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -2615,7 +3383,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -2628,7 +3400,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -2636,7 +3408,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -2649,7 +3425,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -2657,7 +3433,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -2670,7 +3450,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -2678,7 +3458,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -2691,7 +3475,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -2699,7 +3483,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -2712,7 +3500,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -2720,7 +3508,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -2733,7 +3525,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -2741,7 +3533,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -2754,7 +3550,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -2762,7 +3558,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -2775,7 +3575,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -2783,7 +3583,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -2796,7 +3600,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -2804,7 +3608,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -2817,7 +3625,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -2825,7 +3633,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -2838,7 +3650,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -2846,7 +3658,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -2859,7 +3675,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -2867,7 +3683,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -2880,7 +3700,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -2888,7 +3708,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -2901,7 +3725,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -2909,7 +3733,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -2922,7 +3750,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -2930,7 +3758,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -2943,7 +3775,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -2951,7 +3783,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -2964,7 +3800,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -2972,7 +3808,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -2985,7 +3825,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -2993,7 +3833,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -3006,7 +3850,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -3014,7 +3858,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -3027,7 +3875,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -3035,7 +3883,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -3048,7 +3900,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -3056,7 +3908,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -3069,7 +3925,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -3077,7 +3933,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -3090,7 +3950,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>21 June 2026</t>
+          <t>Not Found</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -3098,7 +3958,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -3111,7 +3975,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>12 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -3119,7 +3983,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -3132,7 +4000,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>12 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -3140,7 +4008,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -3153,7 +4025,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>12 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -3161,7 +4033,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr"/>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -3174,7 +4050,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>12 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -3182,7 +4058,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -3195,7 +4075,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -3203,7 +4083,11 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr"/>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -3214,13 +4098,21 @@
           <t>https://doi.org/10.6028/nist.sp.800-88r2</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr"/>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D147" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr"/>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -3231,13 +4123,21 @@
           <t>https://theretroweb.com/storage/documentation/wd6000-velociraptor-68407cb5c0c96653507203.pdf</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr"/>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D148" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -3248,13 +4148,21 @@
           <t>https://www.cyberciti.biz/faq/create-a-freebsd-swap-file/</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr"/>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D149" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr"/>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -3265,13 +4173,21 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=enc</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr"/>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D150" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -3282,13 +4198,21 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=zfs</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr"/>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D151" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr"/>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -3299,13 +4223,21 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=zpool</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr"/>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D152" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr"/>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -3316,13 +4248,21 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=geom</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr"/>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D153" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr"/>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -3333,13 +4273,21 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=geli</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr"/>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D154" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr"/>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -3350,13 +4298,21 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=gpart</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr"/>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D155" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -3367,13 +4323,21 @@
           <t>https://man.freebsd.org/cgi/man.cgi?query=dd</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr"/>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D156" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr"/>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -3384,13 +4348,21 @@
           <t>https://docs.freebsd.org/en/books/handbook/zfs/</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr"/>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D157" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr"/>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -3401,13 +4373,21 @@
           <t>https://docs.freebsd.org/en/books/handbook/disks/</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr"/>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D158" t="inlineStr">
         <is>
           <t>Not Found</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr"/>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>No Wayback Machine snapshot available</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
trying to pull down refs
</commit_message>
<xml_diff>
--- a/KandRStyle/research/references/Reference_Tracking.xlsx
+++ b/KandRStyle/research/references/Reference_Tracking.xlsx
@@ -475,12 +475,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>12 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_001.pdf</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -498,9 +498,14 @@
           <t>http://php.net/manual/en/security.database.sql-injection.php</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_002.pdf</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -518,9 +523,14 @@
           <t>https://owasp.org/index.php/Top</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_003.pdf</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -538,9 +548,14 @@
           <t>https://www.youtube.com/watch?v=uK3\_qR3Kn\_g</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_004.pdf</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -558,9 +573,14 @@
           <t>https://www.scrt.ch/outils/mms/mms</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_005.pdf</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -578,9 +598,14 @@
           <t>https://www.scrt.ch/en/</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_006.pdf</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -598,9 +623,14 @@
           <t>https://www.nist.gov/news-events/events/2017/03/cybersecurity-framework-virtual-events</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_007.pdf</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -618,9 +648,14 @@
           <t>http://faculty.ucmerced.edu/wshadish/shadish-cv-jan-2015</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_008.pdf</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -638,9 +673,14 @@
           <t>http://faculty.ucmerced.edu/wshadish/biosketch</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_009.pdf</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -658,9 +698,14 @@
           <t>http://www.ipr.northwestern.edu/workshops/annual-summer-workshops/quasi-experimental-design-and-analysis/</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_010.pdf</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -678,9 +723,14 @@
           <t>https://www.kali.org/</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_011.pdf</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -698,9 +748,14 @@
           <t>https://www.virtualbox.org/</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_012.pdf</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -718,9 +773,14 @@
           <t>http://www.vmware.com/</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_013.pdf</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -738,9 +798,14 @@
           <t>https://azure.microsoft.com/en-us/?cdn=disable</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_014.pdf</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -758,9 +823,14 @@
           <t>http://junit.org/junit4/</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_015.pdf</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -778,9 +848,14 @@
           <t>http://qunitjs.com/</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_016.pdf</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -798,9 +873,14 @@
           <t>https://phpunit.de/</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_017.pdf</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -818,9 +898,16 @@
           <t>http://docs.seleniumhq.org/</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: net::ERR_NAME_NOT_RESOLVED at http://docs.seleniumhq.org/
+Call log:
+  - navigating to "ht</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -838,9 +925,14 @@
           <t>https://www.microsoft.com/en-us/download/details.aspx?id=3702</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Stored</t>
+          <t>Saved as ref_019.pdf</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -858,9 +950,14 @@
           <t>https://www.mysql.com/</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Timeout - page took too long to load</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -878,9 +975,14 @@
           <t>https://www.phpmyadmin.net/</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_021.pdf</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -898,9 +1000,14 @@
           <t>http://192.168.56.101/chapter4example.exe</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Local/private URL - cannot access</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -918,9 +1025,14 @@
           <t>https://www.owasp.org/index.php/File:Automated-\gls{threat</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_023.pdf</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -938,9 +1050,14 @@
           <t>https://www.youtube.com/watch?v=uK3</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_024.pdf</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -958,9 +1075,14 @@
           <t>http://searchsecurity.techtarget.com/opinion/Wendy-Nather-Were-on-a-trajectory-for-profound-change</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_025.pdf</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -978,9 +1100,14 @@
           <t>http://insecure.org/stf/smashstack.html</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_026.pdf</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -998,9 +1125,14 @@
           <t>http://www.primalsecurity.net/0x0-</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_027.pdf</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1018,9 +1150,14 @@
           <t>https://www.raspberrypi.org/downloads/raspbian/</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Timeout - page took too long to load</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1038,9 +1175,14 @@
           <t>https://docs.kali.org/kali-on-arm/install-kali-linux-arm-raspberry-pi</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_029.pdf</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1058,9 +1200,14 @@
           <t>https://docs.microsoft.com/en-us/powershell/module/microsoft.powershell.utility/get-filehash?view=powershell-5.1</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_030.pdf</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1078,9 +1225,14 @@
           <t>https://unix.stackexchange.com/questions/151547/linux-set-date-through-command-line</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_031.pdf</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1098,9 +1250,14 @@
           <t>https://www.aircrack-ng.org/</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_032.pdf</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1118,9 +1275,14 @@
           <t>https://www.aircrack-ng.org/doku.php?id=compatibility</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_033.pdf</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1138,9 +1300,16 @@
           <t>https://wikidevi.com/wiki/TP-LINK</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: net::ERR_CONNECTION_TIMED_OUT at https://wikidevi.com/wiki/TP-LINK
+Call log:
+  - navigati</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1158,9 +1327,16 @@
           <t>https://wikidevi.com/wiki/ALFA</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t xml:space="preserve">Error: Page.goto: net::ERR_CONNECTION_TIMED_OUT at https://wikidevi.com/wiki/ALFA
+Call log:
+  - navigating </t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1178,9 +1354,14 @@
           <t>https://hakshop.com/products/wifi-pineappling-book</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_036.pdf</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1198,9 +1379,16 @@
           <t>http://goo.gl/iMVWew</t>
         </is>
       </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Download is starting
+Call log:
+  - navigating to "http://goo.gl/iMVWew", waiting until "n</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1218,9 +1406,14 @@
           <t>https://www.raspberrypi.org/</t>
         </is>
       </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_038.pdf</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1238,9 +1431,14 @@
           <t>https://www.raspberrypi.org/documentation/</t>
         </is>
       </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Timeout - page took too long to load</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1258,9 +1456,14 @@
           <t>https://www.walmart.com/ip/TP-LINK-TL-WN722N-N150-High-Gain-Wireless-USB-Adapter/17133249</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Timeout - page took too long to load</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1278,9 +1481,14 @@
           <t>https://www.amazon.com/Alfa-AWUS036NH-802-11g-Wireless-Long-Range/dp/B003YIFHJY</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_041.pdf</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1298,9 +1506,14 @@
           <t>https://www.amazon.com/Alfa-AWUSO36NH-Wireless-Long-Rang-Network/dp/B0035APGP6</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_042.pdf</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1318,9 +1531,14 @@
           <t>https://www.csoonline.com/article/2462478/microsoft-subnet/hacker-hunts-and-pwns-wifi-pineapples-with-0-day-at-def-con.html</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Timeout - page took too long to load</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1338,9 +1556,14 @@
           <t>https://twitter.com/ihuntpineapples/media</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Timeout - page took too long to load</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1358,9 +1581,14 @@
           <t>https://www.reddit.com/r/Defcon/comments/2d16lk/your</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_045.pdf</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1378,9 +1606,14 @@
           <t>https://capec.mitre.org/</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_046.pdf</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1398,9 +1631,14 @@
           <t>https://capec.mitre.org/data/definitions/1000.html</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_047.pdf</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -1418,9 +1656,14 @@
           <t>https://capec.mitre.org/data/definitions/152.html</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_048.pdf</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1438,9 +1681,14 @@
           <t>https://capec.mitre.org/data/definitions/137.html</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_049.pdf</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1458,9 +1706,14 @@
           <t>https://capec.mitre.org/data/definitions/513.html</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_050.pdf</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -1478,9 +1731,14 @@
           <t>https://capec.mitre.org/data/definitions/248.html</t>
         </is>
       </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_051.pdf</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -1498,9 +1756,14 @@
           <t>https://capec.mitre.org/data/definitions/66.html</t>
         </is>
       </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_052.pdf</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -1518,9 +1781,14 @@
           <t>https://capec.mitre.org/data/definitions/108.html</t>
         </is>
       </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_053.pdf</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -1538,9 +1806,14 @@
           <t>http://cwe.mitre.org/data/definitions/707.html</t>
         </is>
       </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_054.pdf</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -1558,9 +1831,14 @@
           <t>http://cwe.mitre.org/data/definitions/74.html</t>
         </is>
       </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_055.pdf</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -1578,9 +1856,14 @@
           <t>http://capec.mitre.org/data/definitions/242.html</t>
         </is>
       </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_056.pdf</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -1598,9 +1881,14 @@
           <t>https://capec.mitre.org/data/definitions/110.html</t>
         </is>
       </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_057.pdf</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -1618,9 +1906,14 @@
           <t>http://cwe.mitre.org/data/definitions/89.html</t>
         </is>
       </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_058.pdf</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -1638,9 +1931,14 @@
           <t>http://cwe.mitre.org/data/definitions/929.html</t>
         </is>
       </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_059.pdf</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -1658,9 +1956,16 @@
           <t>www.linkedin.com/in/derekbrink</t>
         </is>
       </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Protocol error (Page.navigate): Cannot navigate to invalid URL
+Call log:
+  - navigating t</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -1680,12 +1985,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>4 Aug 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_061.pdf</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -1703,9 +2008,14 @@
           <t>https://fred.stlouisfed.org/series/POPTOTASA647NWDB</t>
         </is>
       </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Timeout - page took too long to load</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -1723,9 +2033,14 @@
           <t>https://www.census.gov/quickfacts/chattanoogacitytennessee</t>
         </is>
       </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_063.pdf</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -1743,9 +2058,14 @@
           <t>https://www.census.gov/quickfacts/fact/table/TN/PST045222</t>
         </is>
       </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_064.pdf</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -1763,9 +2083,14 @@
           <t>https://fred.stlouisfed.org/series/CAPOP</t>
         </is>
       </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Timeout - page took too long to load</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -1783,9 +2108,16 @@
           <t>https://www2.census.gov/programs-surveys/popest/datasets/2020-2022/state/totals/NST-EST2022-POPCHG2020_2022.csv</t>
         </is>
       </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Download is starting
+Call log:
+  - navigating to "https://www2.census.gov/programs-survey</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -1803,9 +2135,14 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2016State/StateReport.aspx\#?s=47</t>
         </is>
       </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_067.pdf</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -1823,9 +2160,16 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2016_IC3Report.pdf</t>
         </is>
       </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Download is starting
+Call log:
+  - navigating to "https://www.ic3.gov/AnnualReport/Report</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -1843,9 +2187,14 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2017State/StateReport.aspx\#?s=47</t>
         </is>
       </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_069.pdf</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -1863,9 +2212,16 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2017_IC3Report.pdf</t>
         </is>
       </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Download is starting
+Call log:
+  - navigating to "https://www.ic3.gov/AnnualReport/Report</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -1883,9 +2239,14 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2018State/StateReport.aspx\#?s=47</t>
         </is>
       </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_071.pdf</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -1903,9 +2264,16 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2018_IC3Report.pdf</t>
         </is>
       </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Download is starting
+Call log:
+  - navigating to "https://www.ic3.gov/AnnualReport/Report</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -1923,9 +2291,14 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2019State/StateReport.aspx\#?s=47</t>
         </is>
       </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_073.pdf</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -1943,9 +2316,16 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2019_IC3Report.pdf</t>
         </is>
       </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Download is starting
+Call log:
+  - navigating to "https://www.ic3.gov/AnnualReport/Report</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -1963,9 +2343,14 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2020State/StateReport.aspx\#?s=47</t>
         </is>
       </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_075.pdf</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -1983,9 +2368,16 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2020_IC3Report.pdf</t>
         </is>
       </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Download is starting
+Call log:
+  - navigating to "https://www.ic3.gov/AnnualReport/Report</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -2003,9 +2395,14 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2021State/StateReport.aspx\#?s=47</t>
         </is>
       </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_077.pdf</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -2023,9 +2420,16 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2021_IC3Report.pdf</t>
         </is>
       </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Download is starting
+Call log:
+  - navigating to "https://www.ic3.gov/AnnualReport/Report</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -2043,9 +2447,14 @@
           <t>https://www.ic3.gov/Media/PDF/AnnualReport/2022State/StateReport.aspx\#?s=47</t>
         </is>
       </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Stored</t>
+        </is>
+      </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_079.pdf</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -2063,9 +2472,16 @@
           <t>https://www.ic3.gov/AnnualReport/Reports/2022_IC3Report.pdf</t>
         </is>
       </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Download is starting
+Call log:
+  - navigating to "https://www.ic3.gov/AnnualReport/Report</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -2085,12 +2501,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_081.pdf</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -2110,12 +2526,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_082.pdf</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -2135,12 +2551,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_083.pdf</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -2160,12 +2576,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_084.pdf</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -2185,12 +2601,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_085.pdf</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -2210,12 +2626,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_086.pdf</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -2235,12 +2651,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_087.pdf</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -2260,12 +2676,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_088.pdf</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -2285,12 +2701,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_089.pdf</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -2310,12 +2726,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_090.pdf</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -2335,12 +2751,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_091.pdf</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -2360,12 +2776,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_092.pdf</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -2385,12 +2801,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_093.pdf</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -2410,12 +2826,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_094.pdf</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -2435,12 +2851,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_095.pdf</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -2460,12 +2876,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_096.pdf</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -2485,12 +2901,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_097.pdf</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -2510,12 +2926,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_098.pdf</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -2535,12 +2951,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_099.pdf</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -2560,12 +2976,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_100.pdf</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -2585,12 +3001,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_101.pdf</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -2610,12 +3026,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_102.pdf</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -2635,12 +3051,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_103.pdf</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -2660,12 +3076,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_104.pdf</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -2685,12 +3101,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_105.pdf</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -2710,12 +3126,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_106.pdf</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -2735,12 +3151,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_107.pdf</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -2760,12 +3176,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_108.pdf</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -2785,12 +3201,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_109.pdf</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -2810,12 +3226,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_110.pdf</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -2835,12 +3251,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_111.pdf</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -2860,12 +3276,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_112.pdf</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -2885,12 +3301,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_113.pdf</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -2910,12 +3326,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_114.pdf</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -2935,12 +3351,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_115.pdf</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -2960,12 +3376,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_116.pdf</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -2985,12 +3401,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_117.pdf</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -3010,12 +3426,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_118.pdf</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -3035,12 +3451,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_119.pdf</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -3060,12 +3476,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_120.pdf</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -3085,12 +3501,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_121.pdf</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -3110,12 +3526,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_122.pdf</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -3135,12 +3551,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_123.pdf</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -3160,12 +3576,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_124.pdf</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -3185,12 +3601,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_125.pdf</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -3210,12 +3626,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_126.pdf</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -3235,12 +3651,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_127.pdf</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -3260,12 +3676,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_128.pdf</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -3285,12 +3701,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_129.pdf</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -3310,12 +3726,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_130.pdf</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -3335,12 +3751,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_131.pdf</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -3360,12 +3776,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_132.pdf</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -3385,12 +3801,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_133.pdf</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -3410,12 +3826,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_134.pdf</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -3435,12 +3851,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_135.pdf</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -3460,12 +3876,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_136.pdf</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -3485,12 +3901,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_137.pdf</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -3510,12 +3926,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_138.pdf</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -3535,12 +3951,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_139.pdf</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -3560,12 +3976,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_140.pdf</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -3585,12 +4001,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_141.pdf</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -3610,12 +4026,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>21 June 2026</t>
+          <t>Not Found</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Timeout - page took too long to load</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -3635,12 +4051,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>12 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_143.pdf</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -3660,12 +4076,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>12 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_144.pdf</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -3685,12 +4101,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>12 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_145.pdf</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -3710,12 +4126,12 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>12 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_146.pdf</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -3735,12 +4151,12 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>13 July 2026</t>
+          <t>Stored</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Saved as ref_147.pdf</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -3758,9 +4174,16 @@
           <t>nvlpubs.nist.gov/nistpubs/SpecialPublications/\gls{nist</t>
         </is>
       </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Protocol error (Page.navigate): Cannot navigate to invalid URL
+Call log:
+  - navigating t</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -3778,9 +4201,16 @@
           <t>https://doi.org/10.6028/nist.sp.800-88r2</t>
         </is>
       </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Download is starting
+Call log:
+  - navigating to "https://doi.org/10.6028/nist.sp.800-88r</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -3800,12 +4230,14 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>10 June 2026</t>
+          <t>Not Found</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Protocol error (Page.navigate): Cannot navigate to invalid URL
+Call log:
+  - navigating t</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -3825,12 +4257,14 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>10 June 2026</t>
+          <t>Not Found</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Protocol error (Page.navigate): Cannot navigate to invalid URL
+Call log:
+  - navigating t</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -3848,9 +4282,16 @@
           <t>https://theretroweb.com/storage/documentation/wd6000-velociraptor-68407cb5c0c96653507203.pdf</t>
         </is>
       </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Download is starting
+Call log:
+  - navigating to "https://theretroweb.com/storage/documen</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -3868,9 +4309,16 @@
           <t>www.intel.com/content/dam/doc/product-brief/xeon-5500-server-brief.pdf.</t>
         </is>
       </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Protocol error (Page.navigate): Cannot navigate to invalid URL
+Call log:
+  - navigating t</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -3890,12 +4338,14 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10 June 2026</t>
+          <t>Not Found</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Protocol error (Page.navigate): Cannot navigate to invalid URL
+Call log:
+  - navigating t</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -3913,9 +4363,16 @@
           <t>Docs.oracle.com, docs.oracle.com/cd/E19120-01/open.solaris/817-2271/6mhupg6m3/index.html</t>
         </is>
       </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Protocol error (Page.navigate): Cannot navigate to invalid URL
+Call log:
+  - navigating t</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -3935,12 +4392,14 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>10 June 2026</t>
+          <t>Not Found</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Protocol error (Page.navigate): Cannot navigate to invalid URL
+Call log:
+  - navigating t</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -3960,12 +4419,14 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>10 June 2026</t>
+          <t>Not Found</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Error: Page.goto: Protocol error (Page.navigate): Cannot navigate to invalid URL
+Call log:
+  - navigating t</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">

</xml_diff>